<commit_message>
feat: leitura de codigo de barras
</commit_message>
<xml_diff>
--- a/tests/test_data/teste.xlsx
+++ b/tests/test_data/teste.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="167">
   <si>
     <t>UTE-TL</t>
   </si>
@@ -510,19 +510,31 @@
   <si>
     <t>SIM0029722</t>
   </si>
+  <si>
+    <t>SMIP43753</t>
+  </si>
+  <si>
+    <t>Teste</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -585,13 +597,13 @@
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
@@ -1059,133 +1071,133 @@
       </c>
       <c r="B25" s="5"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75" customFormat="1" s="3">
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="19.5" customFormat="1" s="3">
       <c r="A26" s="4" t="s">
         <v>25</v>
       </c>
       <c r="B26" s="5"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75" customFormat="1" s="3">
+    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="19.5" customFormat="1" s="3">
       <c r="A27" s="4" t="s">
         <v>26</v>
       </c>
       <c r="B27" s="5"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75" customFormat="1" s="3">
+    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="19.5" customFormat="1" s="3">
       <c r="A28" s="4" t="s">
         <v>27</v>
       </c>
       <c r="B28" s="5"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75" customFormat="1" s="3">
+    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="19.5" customFormat="1" s="3">
       <c r="A29" s="4" t="s">
         <v>28</v>
       </c>
       <c r="B29" s="5"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75" customFormat="1" s="3">
+    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="19.5" customFormat="1" s="3">
       <c r="A30" s="4" t="s">
         <v>29</v>
       </c>
       <c r="B30" s="5"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75" customFormat="1" s="3">
+    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="19.5" customFormat="1" s="3">
       <c r="A31" s="4" t="s">
         <v>30</v>
       </c>
       <c r="B31" s="5"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75" customFormat="1" s="3">
+    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="19.5" customFormat="1" s="3">
       <c r="A32" s="4" t="s">
         <v>31</v>
       </c>
       <c r="B32" s="5"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75" customFormat="1" s="3">
+    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="19.5" customFormat="1" s="3">
       <c r="A33" s="4" t="s">
         <v>32</v>
       </c>
       <c r="B33" s="5"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75" customFormat="1" s="3">
+    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="19.5" customFormat="1" s="3">
       <c r="A34" s="4" t="s">
         <v>33</v>
       </c>
       <c r="B34" s="5"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75" customFormat="1" s="3">
+    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="19.5" customFormat="1" s="3">
       <c r="A35" s="4" t="s">
         <v>34</v>
       </c>
       <c r="B35" s="5"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75" customFormat="1" s="3">
+    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="19.5" customFormat="1" s="3">
       <c r="A36" s="4" t="s">
         <v>35</v>
       </c>
       <c r="B36" s="5"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75" customFormat="1" s="3">
+    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="19.5" customFormat="1" s="3">
       <c r="A37" s="4" t="s">
         <v>36</v>
       </c>
       <c r="B37" s="5"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75" customFormat="1" s="3">
+    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="19.5" customFormat="1" s="3">
       <c r="A38" s="4" t="s">
         <v>37</v>
       </c>
       <c r="B38" s="5"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75" customFormat="1" s="3">
+    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="19.5" customFormat="1" s="3">
       <c r="A39" s="4" t="s">
         <v>38</v>
       </c>
       <c r="B39" s="5"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75" customFormat="1" s="3">
+    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="19.5" customFormat="1" s="3">
       <c r="A40" s="4" t="s">
         <v>39</v>
       </c>
       <c r="B40" s="5"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75" customFormat="1" s="3">
+    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="19.5" customFormat="1" s="3">
       <c r="A41" s="4" t="s">
         <v>40</v>
       </c>
       <c r="B41" s="5"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75" customFormat="1" s="3">
+    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="19.5" customFormat="1" s="3">
       <c r="A42" s="4" t="s">
         <v>41</v>
       </c>
       <c r="B42" s="5"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18.75" customFormat="1" s="3">
+    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="19.5" customFormat="1" s="3">
       <c r="A43" s="4" t="s">
         <v>42</v>
       </c>
       <c r="B43" s="5"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="18.75" customFormat="1" s="3">
+    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="19.5" customFormat="1" s="3">
       <c r="A44" s="4" t="s">
         <v>43</v>
       </c>
       <c r="B44" s="5"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18.75" customFormat="1" s="3">
+    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="19.5" customFormat="1" s="3">
       <c r="A45" s="4" t="s">
         <v>44</v>
       </c>
       <c r="B45" s="5"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18.75" customFormat="1" s="3">
+    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="19.5" customFormat="1" s="3">
       <c r="A46" s="4" t="s">
         <v>45</v>
       </c>
       <c r="B46" s="5"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18.75" customFormat="1" s="3">
+    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="19.5" customFormat="1" s="3">
       <c r="A47" s="4" t="s">
         <v>46</v>
       </c>
@@ -1924,8 +1936,12 @@
       <c r="B169" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="170" customHeight="1" ht="18.75" customFormat="1" s="3">
-      <c r="A170" s="8"/>
-      <c r="B170" s="5"/>
+      <c r="A170" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="B170" s="5" t="s">
+        <v>166</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="171" customHeight="1" ht="18.75">
       <c r="A171" s="2"/>

</xml_diff>